<commit_message>
feat(import): mensaje de cruce RN-04 nombra grupo y franja; historico cuenta filas descartadas en preview
</commit_message>
<xml_diff>
--- a/docs/ConIns_ERS_Y_Relevantes/Eventos - ADSO - Agosto - Enviar.xlsx
+++ b/docs/ConIns_ERS_Y_Relevantes/Eventos - ADSO - Agosto - Enviar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\2_ConIns\CONINS_PROJECT_Control_Instructores_SENA\docs\ConIns_ERS_Y_Relevantes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA992C33-F5E3-444B-9A40-846190CB086D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8D658C9-CEFE-4D42-A0BD-9FE5F73CEE97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{D574CE6D-16E2-423B-B366-9F0E7F1F603D}"/>
   </bookViews>
@@ -2518,6 +2518,9 @@
     <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2525,9 +2528,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2884,17 +2884,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="73" t="s">
         <v>77</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
     </row>
     <row r="2" spans="1:10" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
@@ -10533,17 +10533,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="72" t="s">
+      <c r="A1" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="72"/>
-      <c r="C1" s="72"/>
-      <c r="D1" s="72"/>
-      <c r="E1" s="72"/>
-      <c r="F1" s="72"/>
-      <c r="G1" s="72"/>
-      <c r="H1" s="72"/>
-      <c r="I1" s="72"/>
+      <c r="B1" s="73"/>
+      <c r="C1" s="73"/>
+      <c r="D1" s="73"/>
+      <c r="E1" s="73"/>
+      <c r="F1" s="73"/>
+      <c r="G1" s="73"/>
+      <c r="H1" s="73"/>
+      <c r="I1" s="73"/>
     </row>
     <row r="2" spans="1:9" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
@@ -18133,17 +18133,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="73" t="s">
+      <c r="A1" s="74" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="73"/>
-      <c r="C1" s="73"/>
-      <c r="D1" s="73"/>
-      <c r="E1" s="73"/>
-      <c r="F1" s="73"/>
-      <c r="G1" s="73"/>
-      <c r="H1" s="73"/>
-      <c r="I1" s="74"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
+      <c r="D1" s="74"/>
+      <c r="E1" s="74"/>
+      <c r="F1" s="74"/>
+      <c r="G1" s="74"/>
+      <c r="H1" s="74"/>
+      <c r="I1" s="75"/>
     </row>
     <row r="2" spans="1:9" ht="57.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
@@ -26142,17 +26142,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="75" t="s">
+      <c r="A1" s="72" t="s">
         <v>81</v>
       </c>
-      <c r="B1" s="75"/>
-      <c r="C1" s="75"/>
-      <c r="D1" s="75"/>
-      <c r="E1" s="75"/>
-      <c r="F1" s="75"/>
-      <c r="G1" s="75"/>
-      <c r="H1" s="75"/>
-      <c r="I1" s="75"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
+      <c r="D1" s="72"/>
+      <c r="E1" s="72"/>
+      <c r="F1" s="72"/>
+      <c r="G1" s="72"/>
+      <c r="H1" s="72"/>
+      <c r="I1" s="72"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>

</xml_diff>